<commit_message>
Fix Ch.20 reconciliation fixture: align stripe-nov.xlsx outbound payments with the actual 18 invoices (12 matched + 2 partial-pay + 4 unpaid + 1 trap)
</commit_message>
<xml_diff>
--- a/examples/ch-20-finance-ops/stripe-nov.xlsx
+++ b/examples/ch-20-finance-ops/stripe-nov.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00;[Red]-#,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00;-#,##0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -59,9 +60,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,14 +433,14 @@
   <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>py_0000000015</t>
+          <t>py_oct_0001</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -506,7 +509,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Payment to Acme Office Supplies (Oct)</t>
+          <t>Payment to Acme Office Supplies (Oct invoice)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -523,11 +526,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ch_0000000016</t>
+          <t>ch_2001</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45963</v>
+        <v>45962</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -535,7 +538,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>49</v>
+        <v>149</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,12 +547,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
+          <t>Stipendl Pro - monthly subscription</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Customer 8821 - subscription</t>
+          <t>Customer 8821 - Linear Logic LLC</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -561,11 +564,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ch_0000000017</t>
+          <t>ch_2002</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45964</v>
+        <v>45963</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -573,7 +576,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>199</v>
+        <v>299</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -582,12 +585,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Subscription - Team plan</t>
+          <t>Stipendl Team - 5 seats</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Customer 4410 - subscription</t>
+          <t>Customer 1145 - Northwind Holdings</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -599,7 +602,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>st_0000000036</t>
+          <t>ch_2003</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -607,11 +610,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>stripe_fee</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-45.2</v>
+        <v>599</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -620,10 +623,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Stripe processing fees - week 1</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Stipendl Business - 12 seats</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Customer 0033 - Cygnus Robotics</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>succeeded</t>
@@ -633,19 +640,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ch_0000000018</t>
+          <t>fee_4001</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45965</v>
+        <v>45964</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>stripe_fee</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>49</v>
+        <v>-45.2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -654,12 +661,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Customer 9133 - subscription</t>
+          <t>Stripe processing fees - week of Nov 1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -671,7 +673,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ch_0000000019</t>
+          <t>ch_2004</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -683,7 +685,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>99</v>
+        <v>149</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -692,12 +694,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Subscription - Growth plan</t>
+          <t>Stipendl Pro renewal</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Customer 7720 - subscription</t>
+          <t>Customer 2280 - Foundry Health</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -709,7 +711,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>re_0000000033</t>
+          <t>ch_2005</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -717,11 +719,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>refund</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-49</v>
+        <v>1200</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -730,12 +732,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Refund - Pro plan, customer cancel</t>
+          <t>Annual upgrade - Stipendl Business</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Customer 2280 - refund</t>
+          <t>Customer 7720 - Inkpath Studio</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -747,19 +749,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>py_0000000007</t>
+          <t>re_3001</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45968</v>
+        <v>45967</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>refund</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-425.6</v>
+        <v>-49</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -768,12 +770,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Payment to Ridgeway Print</t>
+          <t>Refund - Pro plan, customer cancel within 14d</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Ridgeway Print &amp; Mail</t>
+          <t>Customer 2280 - Foundry Health</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -785,7 +787,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ch_0000000020</t>
+          <t>po_5001</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -793,11 +795,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>payout</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>49</v>
+        <v>-3200</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -806,36 +808,31 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Customer 2280 - subscription</t>
+          <t>Payout to bank ****4421 - week 1 net</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>succeeded</t>
+          <t>paid</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>pa_0000000040</t>
+          <t>py_001</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45968</v>
+        <v>45969</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>payout</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-3200</v>
+        <v>-312.4</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -844,24 +841,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Payout to bank ****4421</t>
+          <t>Payment to Acme Office Supplies</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lumen Analytics Inc</t>
+          <t>Acme Office Supplies Ltd</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>paid</t>
+          <t>succeeded</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>py_0000000001</t>
+          <t>ch_2006</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -869,11 +866,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-312.4</v>
+        <v>299</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -882,12 +879,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Payment to Acme Office Supplies</t>
+          <t>Stipendl Team - 5 seats</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Acme Office Supplies Ltd</t>
+          <t>Customer 4412 - Glacier Capital</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -899,7 +896,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>py_0000000002</t>
+          <t>py_002</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -920,7 +917,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Payment - Brightline Cloud</t>
+          <t>Brightline Cloud Services Nov invoice</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -937,19 +934,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ch_0000000021</t>
+          <t>py_007</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45970</v>
+        <v>45971</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>49</v>
+        <v>-1125</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -958,12 +955,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
+          <t>Marigold Print Workshop - print job</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Customer 5601 - subscription</t>
+          <t>Marigold Print Workshop</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -975,7 +972,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ch_0000000022</t>
+          <t>ch_2007</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -987,7 +984,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>199</v>
+        <v>149</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -996,12 +993,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Subscription - Team plan</t>
+          <t>Stipendl Pro - monthly</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Customer 3344 - subscription</t>
+          <t>Customer 3344 - Banyan Logistics</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1013,7 +1010,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>st_0000000037</t>
+          <t>fee_4002</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1034,10 +1031,9 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Stripe processing fees - week 2</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Stripe processing fees - week of Nov 8</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>succeeded</t>
@@ -1047,19 +1043,19 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>py_0000000013</t>
+          <t>ch_2008</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45972</v>
+        <v>45973</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-2200</v>
+        <v>149</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1068,12 +1064,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Yellowstone Furniture - partial</t>
+          <t>Stipendl Pro - monthly</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yellowstone Furniture Co</t>
+          <t>Customer 9911 - Stoneoak Partners</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1085,11 +1081,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>py_0000000008</t>
+          <t>py_003</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45973</v>
+        <v>45974</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1097,7 +1093,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-1500</v>
+        <v>-4500</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1106,12 +1102,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sable Security - Nov retainer</t>
+          <t>Wire to Halberd Legal - trademark</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Sable Security Services</t>
+          <t>Halberd Legal LLP</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1123,19 +1119,19 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ch_0000000023</t>
+          <t>re_3002</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45973</v>
+        <v>45974</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>refund</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>49</v>
+        <v>-99</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1144,12 +1140,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
+          <t>Refund - duplicate charge investigation</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Customer 8821 - renewal</t>
+          <t>Customer 7720 - Inkpath Studio</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1161,19 +1157,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>re_0000000034</t>
+          <t>py_010p</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45974</v>
+        <v>45975</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>refund</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>-99</v>
+        <v>-2500</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1182,12 +1178,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Refund - dispute resolved</t>
+          <t>Saffron Recruitment - 1st instalment of staged retainer</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Customer 7720 - refund</t>
+          <t>Saffron Recruitment Partners</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1199,7 +1195,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ch_0000000024</t>
+          <t>ch_2009</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -1211,7 +1207,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1220,12 +1216,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Subscription - Scale plan</t>
+          <t>Stipendl Business - 12 seats</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Customer 6612 - subscription</t>
+          <t>Customer 5512 - Polar Forge GmbH</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1237,7 +1233,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>pa_0000000041</t>
+          <t>po_5002</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1258,12 +1254,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Payout to bank ****4421</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Lumen Analytics Inc</t>
+          <t>Payout to bank ****4421 - week 2 net</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1275,7 +1266,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>py_0000000004</t>
+          <t>py_004</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -1296,7 +1287,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Pinewood Coworking Nov membership</t>
+          <t>Pinewood Coworking November</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1313,11 +1304,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ch_0000000025</t>
+          <t>ch_2010</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45976</v>
+        <v>45978</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1325,7 +1316,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>99</v>
+        <v>299</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1334,12 +1325,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Subscription - Growth plan</t>
+          <t>Stipendl Team - 5 seats</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Customer 1145 - subscription</t>
+          <t>Customer 6677 - Aurelius Trading</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1351,19 +1342,19 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ch_0000000044</t>
+          <t>fee_4003</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45977</v>
+        <v>45978</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>stripe_fee</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>49</v>
+        <v>-48.1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1372,28 +1363,23 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Customer 4502 - subscription</t>
+          <t>Stripe processing fees - week of Nov 15</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>failed</t>
+          <t>succeeded</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ch_0000000026</t>
+          <t>ch_2011</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45978</v>
+        <v>45979</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1401,7 +1387,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>49</v>
+        <v>149</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1410,12 +1396,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
+          <t>Stipendl Pro - monthly</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Customer 9988 - subscription</t>
+          <t>Customer 8821 - Linear Logic LLC</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1427,19 +1413,19 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>st_0000000038</t>
+          <t>py_012</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45978</v>
+        <v>45980</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>stripe_fee</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-48.1</v>
+        <v>-3300</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1448,10 +1434,14 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Stripe processing fees - week 3</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>Veridian Labs - November subscription</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Veridian Labs</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>succeeded</t>
@@ -1461,19 +1451,19 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>py_0000000009</t>
+          <t>ch_6001</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45979</v>
+        <v>45980</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>-3200</v>
+        <v>599</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1482,28 +1472,28 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Tidepool Consulting Nov</t>
+          <t>Stipendl Business - retry next cycle</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Tidepool Consulting</t>
+          <t>Customer 5599 - Cobalt Networks</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>succeeded</t>
+          <t>failed</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ch_0000000027</t>
+          <t>ch_2012</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45980</v>
+        <v>45981</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1511,7 +1501,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>199</v>
+        <v>149</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1520,12 +1510,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Subscription - Team plan</t>
+          <t>Stipendl Pro - monthly</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Customer 3344 - upgrade</t>
+          <t>Customer 4499 - Tundra Foods Co</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1537,11 +1527,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>py_0000000003</t>
+          <t>py_005</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45981</v>
+        <v>45982</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1549,7 +1539,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>-4500</v>
+        <v>-6750</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1558,12 +1548,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Wire to Halberd Legal</t>
+          <t>Tessera Design Studio brand refresh</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Halberd Legal LLP</t>
+          <t>Tessera Design Studio</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1575,7 +1565,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ch_0000000028</t>
+          <t>po_5003</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -1583,11 +1573,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>payout</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>49</v>
+        <v>-3100</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1596,62 +1586,57 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Customer 7401 - subscription</t>
+          <t>Payout to bank ****4421 - week 3 net</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>succeeded</t>
+          <t>paid</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>pa_0000000042</t>
+          <t>py_013</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45982</v>
+        <v>45983</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>payout</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>-3100</v>
+        <v>-1485</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Payout to bank ****4421</t>
+          <t>Aster Holdings - consulting (SGD)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Lumen Analytics Inc</t>
+          <t>Aster Holdings Pte Ltd</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>paid</t>
+          <t>succeeded</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>py_0000000010</t>
+          <t>py_014p</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
@@ -1663,7 +1648,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-980</v>
+        <v>-2500</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1672,12 +1657,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Umbra Translation - JP localization</t>
+          <t>Mercer Group - partial payment (balance to follow)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Umbra Translation Co</t>
+          <t>Mercer Group</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1689,7 +1674,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ch_0000000029</t>
+          <t>ch_2013</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1701,7 +1686,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>49</v>
+        <v>299</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1710,12 +1695,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
+          <t>Stipendl Team - 5 seats</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Customer 1212 - subscription</t>
+          <t>Customer 1077 - Marlowe Studio</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1727,7 +1712,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>re_0000000035</t>
+          <t>re_3003</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -1739,7 +1724,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>-199</v>
+        <v>-240</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1748,12 +1733,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Refund - duplicate charge</t>
+          <t>Refund - misapplied annual upgrade</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Customer 3344 - refund</t>
+          <t>Customer 1077 - Marlowe Studio</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1765,7 +1750,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>py_0000000005</t>
+          <t>ch_2014</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1773,11 +1758,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>-6750</v>
+        <v>599</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1786,12 +1771,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Tessera Design - brand phase 2</t>
+          <t>Stipendl Business - 12 seats</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tessera Design Studio</t>
+          <t>Customer 2200 - Halo Diagnostics</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1803,7 +1788,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ch_0000000030</t>
+          <t>fee_4004</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
@@ -1811,11 +1796,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>stripe_fee</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>99</v>
+        <v>-41.9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1824,12 +1809,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Subscription - Growth plan</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Customer 8855 - subscription</t>
+          <t>Stripe processing fees - week of Nov 22</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1841,19 +1821,19 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>st_0000000039</t>
+          <t>py_015</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45985</v>
+        <v>45986</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>stripe_fee</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>-41.9</v>
+        <v>-1000</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1862,10 +1842,14 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Stripe processing fees - week 4</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>Sunfield Bakery - office event catering</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Sunfield Bakery</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>succeeded</t>
@@ -1875,11 +1859,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>py_0000000011</t>
+          <t>py_016</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45986</v>
+        <v>45987</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1887,7 +1871,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>-5400</v>
+        <v>-3440</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1896,12 +1880,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Verity Audit - Q3 review</t>
+          <t>Halcyon Studios - product photography</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Verity Audit Partners</t>
+          <t>Halcyon Studios</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1913,19 +1897,19 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>py_0000000006</t>
+          <t>ch_2015</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45987</v>
+        <v>45988</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>-890</v>
+        <v>149</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1934,12 +1918,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Northgate Catering - offsite</t>
+          <t>Stipendl Pro - monthly</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Northgate Catering Co</t>
+          <t>Customer 3318 - Beacon &amp; Co</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1951,19 +1935,19 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ch_0000000031</t>
+          <t>py_017</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45987</v>
+        <v>45989</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>charge</t>
+          <t>payment</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>49</v>
+        <v>-4120</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1972,12 +1956,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Subscription - Pro plan</t>
+          <t>Pine &amp; Co - audit fieldwork Nov</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Customer 6712 - subscription</t>
+          <t>Pine &amp; Co</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -1989,19 +1973,19 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>py_0000000012</t>
+          <t>po_5004</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45988</v>
+        <v>45989</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>payout</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>-2860</v>
+        <v>-2950</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2010,28 +1994,23 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Westwind Travel - offsite flights</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Westwind Travel Agency</t>
+          <t>Payout to bank ****4421 - week 4 net</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>succeeded</t>
+          <t>paid</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>py_0000000014</t>
+          <t>py_018</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -2039,7 +2018,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>-3900</v>
+        <v>-816</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2048,12 +2027,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Zenith Software - partial pmt</t>
+          <t>Blue Harbor Cafe - team lunches November</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Zenith Software Labs</t>
+          <t>Blue Harbor Cafe</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2065,11 +2044,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ch_0000000032</t>
+          <t>ch_2016</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45989</v>
+        <v>45990</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -2077,7 +2056,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>199</v>
+        <v>299</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2086,12 +2065,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Subscription - Team plan</t>
+          <t>Stipendl Team - 5 seats</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Customer 9090 - subscription</t>
+          <t>Customer 8866 - Reverb Audio Inc</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2103,19 +2082,19 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>pa_0000000043</t>
+          <t>ch_2017</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45989</v>
+        <v>45991</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>payout</t>
+          <t>charge</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>-2950</v>
+        <v>149</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2124,17 +2103,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Payout to bank ****4421</t>
+          <t>Stipendl Pro - monthly</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Lumen Analytics Inc</t>
+          <t>Customer 1010 - Quanta Microsystems</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>paid</t>
+          <t>succeeded</t>
         </is>
       </c>
     </row>

</xml_diff>